<commit_message>
Integracion a la intranet
</commit_message>
<xml_diff>
--- a/Registros/Plantillas/Call Center/Plantillas CC.xlsx
+++ b/Registros/Plantillas/Call Center/Plantillas CC.xlsx
@@ -5,21 +5,21 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/69517450a5f14e94/Intranet/Secciones Pendientes y Proyectos/Registros/Plantillas/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/69517450a5f14e94/Intranet/Registros/Plantillas/Call Center/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="262" documentId="8_{CBCA95D9-4624-45FE-A3AD-1F8F82757BF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C7FD0D15-1747-4462-92CF-32DE69A3ED18}"/>
+  <xr:revisionPtr revIDLastSave="263" documentId="8_{CBCA95D9-4624-45FE-A3AD-1F8F82757BF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{448BCDE2-C8BC-4BA5-AB0C-425D486D7FF0}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="7" activeTab="7" xr2:uid="{8F7AADFA-65C7-4638-B903-4D5A4DA683E7}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="2" activeTab="6" xr2:uid="{8F7AADFA-65C7-4638-B903-4D5A4DA683E7}"/>
   </bookViews>
   <sheets>
-    <sheet name="Falla de Voz" sheetId="1" state="hidden" r:id="rId1"/>
-    <sheet name="Falla de Navegacion" sheetId="2" state="hidden" r:id="rId2"/>
-    <sheet name="Falla Total" sheetId="4" state="hidden" r:id="rId3"/>
-    <sheet name="Recargas" sheetId="5" state="hidden" r:id="rId4"/>
-    <sheet name="Callback" sheetId="6" state="hidden" r:id="rId5"/>
-    <sheet name="Migracion" sheetId="7" state="hidden" r:id="rId6"/>
-    <sheet name="Seguimiento a correo" sheetId="8" state="hidden" r:id="rId7"/>
+    <sheet name="Falla de Voz" sheetId="1" r:id="rId1"/>
+    <sheet name="Falla de Navegacion" sheetId="2" r:id="rId2"/>
+    <sheet name="Falla Total" sheetId="4" r:id="rId3"/>
+    <sheet name="Recargas" sheetId="5" r:id="rId4"/>
+    <sheet name="Callback" sheetId="6" r:id="rId5"/>
+    <sheet name="Migracion" sheetId="7" r:id="rId6"/>
+    <sheet name="Seguimiento a correo" sheetId="8" r:id="rId7"/>
     <sheet name="Reactivacion" sheetId="9" r:id="rId8"/>
     <sheet name="Informacion" sheetId="3" r:id="rId9"/>
     <sheet name="Otros" sheetId="10" r:id="rId10"/>
@@ -853,10 +853,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>